<commit_message>
Home hero in the Handbook cover palette; Handbook view toggle
- Hero: navy field closed by horizontal chevron bands in the cover colours; the chevron
  point leans toward the cursor, bands bulge around it, packets run along the seams
- Handbook reader has no add buttons by default; "Use Handbook view" (builder intro and
  header) turns them on for the session, with a bar to go back or turn it off
- Handbook intro: Betsy's edits (Build an Agreement as the way to assemble)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Digital Ceasefire Platform.xlsx
+++ b/Digital Ceasefire Platform.xlsx
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>The full text of the Digital Ceasefire &amp; De-escalation Handbook is available here, section by section, or it can be downloaded in full in [PDF format](#handbook-pdf). The Handbook guides users through the process of developing an Agreement, either by selecting appropriate provisions of the Handbook into an Agreement or by using the Platform's [Build an Agreement function](#/builder). We recommend starting with reading the [Note to Users](#/handbook/s-note-to-users) below. Sections 1.0 through 11.0 then provide model provisions that can be selected, adapted, and combined to construct an Agreement tailored to different conflict and security contexts.</t>
+          <t>The full text of the Digital Ceasefire &amp; De-escalation Handbook is available here, section by section, or it can be downloaded in full in [PDF format](#handbook-pdf). The Handbook guides users through the process of developing an Agreement, using the Platform's [Build an Agreement function](#/builder). We recommend starting with reading the [Note to Users](#/handbook/s-note-to-users) below. Sections 1.0 through 11.0 then provide model provisions that can be selected, adapted, and combined in [Build an Agreement](#/builder) to construct an Agreement tailored to different conflict and security contexts.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1165,7 +1165,7 @@
 To get started, choose one of three approaches:
 - **Build from scratch:** Select the provisions you wish to include from the left-hand column and add them to your Agreement in the right-hand column.
 - **Start with the full Agreement:** Add all of the Handbook's model provisions to your Agreement, then remove those that are not relevant.
-- **Use the Handbook:** Read the [Handbook](#/handbook) section by section and add provisions to your Agreement as you go.
+- **Use Handbook view:** Read the Handbook section by section and add provisions to your Agreement as you go.
 Either way, once you have selected your provisions, you can edit and adapt the text in the right-hand column to reflect the specific circumstances, priorities, and commitments of the Parties.
 Your Agreement is saved automatically in this browser, and you can come back to it at any time. You will find your saved Agreements in the Drafts box at the top left of the builder.
 You can download your Agreement in various formats: Word, Markdown and PDF, by selecting the format in the Export drop down.

</xml_diff>

<commit_message>
Drop utm_source=chatgpt.com from footnote 79 link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Digital Ceasefire Platform.xlsx
+++ b/Digital Ceasefire Platform.xlsx
@@ -20919,12 +20919,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>OECD Legal Instruments, Recommendation of the Council on Information Integrity, https://legalinstruments.oecd.org/en/instruments/OECD-LEGAL-0505?trk=article-ssr-frontend-pulse_little-text-block&amp;utm_source=chatgpt.com.</t>
+          <t>OECD Legal Instruments, Recommendation of the Council on Information Integrity, https://legalinstruments.oecd.org/en/instruments/OECD-LEGAL-0505?trk=article-ssr-frontend-pulse_little-text-block.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://legalinstruments.oecd.org/en/instruments/OECD-LEGAL-0505?trk=article-ssr-frontend-pulse_little-text-block&amp;utm_source=chatgpt.com</t>
+          <t>https://legalinstruments.oecd.org/en/instruments/OECD-LEGAL-0505?trk=article-ssr-frontend-pulse_little-text-block</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop remaining utm_source=chatgpt.com from footnote links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Digital Ceasefire Platform.xlsx
+++ b/Digital Ceasefire Platform.xlsx
@@ -20282,7 +20282,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Organisation for Economic Co-operation and Development (OECD), Explanatory Memorandum on the Updated OECD Definition of an AI System, OECD Artificial Intelligence Papers, no. 8 (Paris: OECD Publishing, 2024), 4, [https://doi.org/10.1787/623da898-en](https://doi.org/10.1787/623da898-en?utm_source=chatgpt.com).</t>
+          <t>Organisation for Economic Co-operation and Development (OECD), Explanatory Memorandum on the Updated OECD Definition of an AI System, OECD Artificial Intelligence Papers, no. 8 (Paris: OECD Publishing, 2024), 4, [https://doi.org/10.1787/623da898-en](https://doi.org/10.1787/623da898-en).</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -21306,7 +21306,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>See *Legality of the Threat or Use of Nuclear Weapons*, Advisory Opinion, July 8, 1996, *I.C.J. Reports* 1996, 226, 244, ¶ 39, [https://www.icj-cij.org/case/95/advisory-opinions](https://www.icj-cij.org/case/95/advisory-opinions?utm_source=chatgpt.com) (providing that Articles 2(4) and 51 “do not refer to specific weapons” and “apply to any use of force, regardless of the weapons employed”).</t>
+          <t>See *Legality of the Threat or Use of Nuclear Weapons*, Advisory Opinion, July 8, 1996, *I.C.J. Reports* 1996, 226, 244, ¶ 39, [https://www.icj-cij.org/case/95/advisory-opinions](https://www.icj-cij.org/case/95/advisory-opinions) (providing that Articles 2(4) and 51 “do not refer to specific weapons” and “apply to any use of force, regardless of the weapons employed”).</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">

</xml_diff>